<commit_message>
updated step overlap and tests
</commit_message>
<xml_diff>
--- a/i_test/05_04_test_reconciliation_2/i_input_xls/D3_pregnancy_model.xlsx
+++ b/i_test/05_04_test_reconciliation_2/i_input_xls/D3_pregnancy_model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giorg\GitHub\ConcePTIONAlgorithmPregnancies\i_test\05_04_test_reconciliation_2\i_input_xls\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AD8287-12DA-4E4B-B485-10A892A98988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0641FF04-227C-4156-A80E-2E7CEF775C99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{D1A11112-67A8-475A-9188-334D63078A0E}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{D1A11112-67A8-475A-9188-334D63078A0E}"/>
   </bookViews>
   <sheets>
     <sheet name="D3_pregnancy_model" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>pregnancy_id</t>
   </si>
@@ -80,6 +80,12 @@
   </si>
   <si>
     <t>3_blue</t>
+  </si>
+  <si>
+    <t>algorithm_for_reconciliation</t>
+  </si>
+  <si>
+    <t>x</t>
   </si>
 </sst>
 </file>
@@ -961,24 +967,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F82B6EA-E582-41B0-961C-9FF974296178}">
-  <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.5546875" customWidth="1"/>
-    <col min="12" max="12" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1015,8 +1021,11 @@
       <c r="L1" t="s">
         <v>15</v>
       </c>
+      <c r="M1" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1053,8 +1062,11 @@
       <c r="L2" t="s">
         <v>16</v>
       </c>
+      <c r="M2" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1091,8 +1103,11 @@
       <c r="L3" t="s">
         <v>19</v>
       </c>
+      <c r="M3" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1128,6 +1143,9 @@
       </c>
       <c r="L4" t="s">
         <v>17</v>
+      </c>
+      <c r="M4" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>